<commit_message>
Upload all the new scripts and files
</commit_message>
<xml_diff>
--- a/MAPE.xlsx
+++ b/MAPE.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\priip\Documents\repos\selec_mondelez\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASSURANCE IT\repos\projects\mdlz-selec\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667EF07F-B7F7-45F9-AC0E-9195E49253B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9FE09E5-8087-435F-82A6-973D0C7513BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12816" xr2:uid="{3532AA99-C125-4593-B349-FFA9325669F7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{3532AA99-C125-4593-B349-FFA9325669F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
-    <sheet name="Planilha2" sheetId="2" r:id="rId2"/>
+    <sheet name="Planilha4" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="81">
   <si>
     <t>Cereal Bar 50g</t>
   </si>
@@ -118,27 +118,6 @@
     <t>MAPE_v5</t>
   </si>
   <si>
-    <t>mape</t>
-  </si>
-  <si>
-    <t>wmape</t>
-  </si>
-  <si>
-    <t>mae</t>
-  </si>
-  <si>
-    <t>rmse</t>
-  </si>
-  <si>
-    <t>n_semanas</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>ok</t>
-  </si>
-  <si>
     <t>Resultado</t>
   </si>
   <si>
@@ -157,15 +136,6 @@
     <t>v6</t>
   </si>
   <si>
-    <t>cv_mape</t>
-  </si>
-  <si>
-    <t>best_params</t>
-  </si>
-  <si>
-    <t>{'subsample_freq': 1, 'boosting_type': 'gbdt',,,,</t>
-  </si>
-  <si>
     <t>MAPE_v6</t>
   </si>
   <si>
@@ -179,13 +149,133 @@
   </si>
   <si>
     <t>Substituido o método de Random Search por Optmun, para seleção de hiperparametros</t>
+  </si>
+  <si>
+    <t>Metodo</t>
+  </si>
+  <si>
+    <t>Constraint</t>
+  </si>
+  <si>
+    <t>Modelo</t>
+  </si>
+  <si>
+    <t>Accuracy_Atual_%</t>
+  </si>
+  <si>
+    <t>Accuracy_Baseline_%</t>
+  </si>
+  <si>
+    <t>Delta_pp</t>
+  </si>
+  <si>
+    <t>Energy Drink</t>
+  </si>
+  <si>
+    <t>Pooling</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>LightGBM</t>
+  </si>
+  <si>
+    <t>Whole Grain Crackers</t>
+  </si>
+  <si>
+    <t>SKU-level</t>
+  </si>
+  <si>
+    <t>Nao</t>
+  </si>
+  <si>
+    <t>Flavored Water</t>
+  </si>
+  <si>
+    <t>XGBoost</t>
+  </si>
+  <si>
+    <t>Cereal Bar</t>
+  </si>
+  <si>
+    <t>GAM</t>
+  </si>
+  <si>
+    <t>Natural Juice</t>
+  </si>
+  <si>
+    <t>59,8</t>
+  </si>
+  <si>
+    <t>23,3</t>
+  </si>
+  <si>
+    <t>22,5</t>
+  </si>
+  <si>
+    <t>6,3</t>
+  </si>
+  <si>
+    <t>5,2</t>
+  </si>
+  <si>
+    <t>1,9</t>
+  </si>
+  <si>
+    <t>1,5</t>
+  </si>
+  <si>
+    <t>0,2</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>INSTAVEL -- accuracy negativa, risco de dado nao resolvido</t>
+  </si>
+  <si>
+    <t>LightGBM Tuned</t>
+  </si>
+  <si>
+    <t>Decisao pendente</t>
+  </si>
+  <si>
+    <t>LightGBM (tuned)</t>
+  </si>
+  <si>
+    <t>Trocado de Stacked p/ GAM (stacked nao fechou a restricao)</t>
+  </si>
+  <si>
+    <t>30,7</t>
+  </si>
+  <si>
+    <t>C/ constraint = 64,2% (-4,7pp) | S/ constraint = 69,0%</t>
+  </si>
+  <si>
+    <t>12,7</t>
+  </si>
+  <si>
+    <t>1,8</t>
+  </si>
+  <si>
+    <t>1,3</t>
+  </si>
+  <si>
+    <t>0,8</t>
+  </si>
+  <si>
+    <t>-0,1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -194,6 +284,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -222,12 +327,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -544,15 +664,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D93C970-6581-46E7-A70C-2DD1017BCA62}">
   <dimension ref="B2:T29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.88671875" style="1"/>
+    <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
         <v>3</v>
       </c>
@@ -590,22 +710,22 @@
         <v>20</v>
       </c>
       <c r="O2" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="P2" t="s">
         <v>20</v>
       </c>
       <c r="Q2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="R2" t="s">
         <v>20</v>
       </c>
       <c r="S2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>0</v>
       </c>
@@ -672,7 +792,7 @@
         <v>0.87728799999999996</v>
       </c>
     </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>1</v>
       </c>
@@ -733,7 +853,7 @@
         <v>-0.20386199999999999</v>
       </c>
     </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>2</v>
       </c>
@@ -794,7 +914,7 @@
         <v>6.2713000000000019E-2</v>
       </c>
     </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>3</v>
       </c>
@@ -855,7 +975,7 @@
         <v>1.6252000000000044E-2</v>
       </c>
     </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>4</v>
       </c>
@@ -916,7 +1036,7 @@
         <v>0.86214100000000005</v>
       </c>
     </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>5</v>
       </c>
@@ -977,7 +1097,7 @@
         <v>0.76499499999999998</v>
       </c>
     </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>6</v>
       </c>
@@ -1038,7 +1158,7 @@
         <v>0.70240900000000006</v>
       </c>
     </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>7</v>
       </c>
@@ -1099,7 +1219,7 @@
         <v>0.72268399999999999</v>
       </c>
     </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>8</v>
       </c>
@@ -1160,7 +1280,7 @@
         <v>0.74879099999999998</v>
       </c>
     </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>9</v>
       </c>
@@ -1221,7 +1341,7 @@
         <v>0.73414899999999994</v>
       </c>
     </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>10</v>
       </c>
@@ -1282,7 +1402,7 @@
         <v>0.68256600000000001</v>
       </c>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>11</v>
       </c>
@@ -1343,7 +1463,7 @@
         <v>0.79152699999999998</v>
       </c>
     </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>12</v>
       </c>
@@ -1404,7 +1524,7 @@
         <v>0.73785499999999993</v>
       </c>
     </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>13</v>
       </c>
@@ -1465,7 +1585,7 @@
         <v>0.75350399999999995</v>
       </c>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>14</v>
       </c>
@@ -1526,7 +1646,7 @@
         <v>0.54833799999999999</v>
       </c>
     </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="E18">
         <f>AVERAGE(E3:E17)</f>
         <v>45.17133333333333</v>
@@ -1561,7 +1681,7 @@
         <v>0.58675666666666648</v>
       </c>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>14</v>
       </c>
@@ -1572,10 +1692,10 @@
         <v>16</v>
       </c>
       <c r="F21" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
         <v>12</v>
       </c>
@@ -1586,7 +1706,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
         <v>18</v>
       </c>
@@ -1594,7 +1714,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C24" t="s">
         <v>21</v>
       </c>
@@ -1602,7 +1722,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
         <v>24</v>
       </c>
@@ -1610,7 +1730,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
         <v>27</v>
       </c>
@@ -1618,31 +1738,31 @@
         <v>28</v>
       </c>
       <c r="F26" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="C28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D28" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="C29" t="s">
-        <v>49</v>
-      </c>
-      <c r="D29" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1652,570 +1772,475 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F3EFF46-E95F-4FFA-BAB5-1DCE8A572C39}">
-  <dimension ref="C3:M18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A96E91DB-06F2-46D4-B4A8-214070126B2F}">
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="55.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="D3" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E3" t="s">
+      <c r="B1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" t="s">
-        <v>32</v>
-      </c>
-      <c r="I3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="C1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="K3" t="s">
-        <v>34</v>
-      </c>
-      <c r="L3" t="s">
-        <v>35</v>
-      </c>
-      <c r="M3" t="s">
+      <c r="F1" s="6" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="4" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C4">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="G1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F4">
-        <v>0.122712</v>
-      </c>
-      <c r="G4">
-        <v>0.119238</v>
-      </c>
-      <c r="H4">
-        <v>0.118149</v>
-      </c>
-      <c r="I4">
-        <v>0.14960599999999999</v>
-      </c>
-      <c r="J4">
-        <v>0.11158999999999999</v>
-      </c>
-      <c r="K4">
-        <v>156</v>
-      </c>
-      <c r="L4" t="s">
-        <v>36</v>
-      </c>
-      <c r="M4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="C2" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" s="6">
+        <v>85</v>
+      </c>
+      <c r="G2" s="8">
+        <v>79.8</v>
+      </c>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F5">
-        <v>1.203862</v>
-      </c>
-      <c r="G5">
-        <v>0.54205300000000001</v>
-      </c>
-      <c r="H5">
-        <v>0.780528</v>
-      </c>
-      <c r="I5">
-        <v>0.95151799999999997</v>
-      </c>
-      <c r="J5">
-        <v>0.67618999999999996</v>
-      </c>
-      <c r="K5">
-        <v>156</v>
-      </c>
-      <c r="L5" t="s">
-        <v>36</v>
-      </c>
-      <c r="M5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="C3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="7">
+        <v>-19</v>
+      </c>
+      <c r="G3" s="9">
+        <v>-78.8</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F6">
-        <v>0.93728699999999998</v>
-      </c>
-      <c r="G6">
-        <v>0.49829699999999999</v>
-      </c>
-      <c r="H6">
-        <v>0.90929599999999999</v>
-      </c>
-      <c r="I6">
-        <v>1.160039</v>
-      </c>
-      <c r="J6">
-        <v>0.71476200000000001</v>
-      </c>
-      <c r="K6">
-        <v>156</v>
-      </c>
-      <c r="L6" t="s">
-        <v>36</v>
-      </c>
-      <c r="M6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C7">
+      <c r="C4" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="7">
+        <v>-30.6</v>
+      </c>
+      <c r="G4" s="9">
+        <v>-53.9</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="C5" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="6">
+        <v>69</v>
+      </c>
+      <c r="G5" s="8">
+        <v>56.3</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F7">
-        <v>0.98374799999999996</v>
-      </c>
-      <c r="G7">
-        <v>0.51851000000000003</v>
-      </c>
-      <c r="H7">
-        <v>1.141413</v>
-      </c>
-      <c r="I7">
-        <v>1.4219569999999999</v>
-      </c>
-      <c r="J7">
-        <v>0.97192500000000004</v>
-      </c>
-      <c r="K7">
-        <v>156</v>
-      </c>
-      <c r="L7" t="s">
-        <v>36</v>
-      </c>
-      <c r="M7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C8">
-        <v>13</v>
-      </c>
-      <c r="D8" t="s">
-        <v>7</v>
-      </c>
-      <c r="E8" t="s">
-        <v>1</v>
-      </c>
-      <c r="F8">
-        <v>0.13785900000000001</v>
-      </c>
-      <c r="G8">
-        <v>0.13131300000000001</v>
-      </c>
-      <c r="H8">
-        <v>0.12873399999999999</v>
-      </c>
-      <c r="I8">
-        <v>0.16138</v>
-      </c>
-      <c r="J8">
-        <v>0.148066</v>
-      </c>
-      <c r="K8">
-        <v>156</v>
-      </c>
-      <c r="L8" t="s">
-        <v>36</v>
-      </c>
-      <c r="M8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="9" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C9">
-        <v>11</v>
-      </c>
-      <c r="D9" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="C6" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="6">
+        <v>79.599999999999994</v>
+      </c>
+      <c r="G6" s="8">
+        <v>78.099999999999994</v>
+      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F9">
-        <v>0.23500499999999999</v>
-      </c>
-      <c r="G9">
-        <v>0.21538499999999999</v>
-      </c>
-      <c r="H9">
-        <v>0.54995099999999997</v>
-      </c>
-      <c r="I9">
-        <v>0.70358100000000001</v>
-      </c>
-      <c r="J9">
-        <v>0.192436</v>
-      </c>
-      <c r="K9">
-        <v>156</v>
-      </c>
-      <c r="L9" t="s">
-        <v>36</v>
-      </c>
-      <c r="M9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C10">
-        <v>5</v>
-      </c>
-      <c r="D10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="C7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="6">
+        <v>78.2</v>
+      </c>
+      <c r="G7" s="8">
+        <v>78.099999999999994</v>
+      </c>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F10">
-        <v>0.29759099999999999</v>
-      </c>
-      <c r="G10">
-        <v>0.23711199999999999</v>
-      </c>
-      <c r="H10">
-        <v>1.0351539999999999</v>
-      </c>
-      <c r="I10">
-        <v>1.3027230000000001</v>
-      </c>
-      <c r="J10">
-        <v>0.27953699999999998</v>
-      </c>
-      <c r="K10">
-        <v>156</v>
-      </c>
-      <c r="L10" t="s">
-        <v>36</v>
-      </c>
-      <c r="M10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C11">
-        <v>6</v>
-      </c>
-      <c r="D11" t="s">
-        <v>5</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="C8" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="6">
+        <v>77.900000000000006</v>
+      </c>
+      <c r="G8" s="8">
+        <v>77.7</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F11">
-        <v>0.27731600000000001</v>
-      </c>
-      <c r="G11">
-        <v>0.243029</v>
-      </c>
-      <c r="H11">
-        <v>1.271922</v>
-      </c>
-      <c r="I11">
-        <v>1.5823780000000001</v>
-      </c>
-      <c r="J11">
-        <v>0.31443199999999999</v>
-      </c>
-      <c r="K11">
-        <v>156</v>
-      </c>
-      <c r="L11" t="s">
-        <v>36</v>
-      </c>
-      <c r="M11" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C12">
+      <c r="C9" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="6">
+        <v>66.5</v>
+      </c>
+      <c r="G9" s="8">
+        <v>66.599999999999994</v>
+      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="6">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="G10" s="8">
+        <v>68.599999999999994</v>
+      </c>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" s="6">
+        <v>79.3</v>
+      </c>
+      <c r="G11" s="8">
+        <v>77.5</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D12" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12">
-        <v>0.25120900000000002</v>
-      </c>
-      <c r="G12">
-        <v>0.22228600000000001</v>
-      </c>
-      <c r="H12">
-        <v>1.670936</v>
-      </c>
-      <c r="I12">
-        <v>2.2613759999999998</v>
-      </c>
-      <c r="J12">
-        <v>0.23662900000000001</v>
-      </c>
-      <c r="K12">
-        <v>156</v>
-      </c>
-      <c r="L12" t="s">
-        <v>36</v>
-      </c>
-      <c r="M12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C13">
-        <v>7</v>
-      </c>
-      <c r="D13" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13">
-        <v>0.265851</v>
-      </c>
-      <c r="G13">
-        <v>0.22542499999999999</v>
-      </c>
-      <c r="H13">
-        <v>0.66085700000000003</v>
-      </c>
-      <c r="I13">
-        <v>0.80679900000000004</v>
-      </c>
-      <c r="J13">
-        <v>0.20121</v>
-      </c>
-      <c r="K13">
-        <v>156</v>
-      </c>
-      <c r="L13" t="s">
-        <v>36</v>
-      </c>
-      <c r="M13" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="14" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C14">
-        <v>4</v>
-      </c>
-      <c r="D14" t="s">
-        <v>0</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="C12" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F12" s="6">
+        <v>60</v>
+      </c>
+      <c r="G12" s="8">
+        <v>37.5</v>
+      </c>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F14">
-        <v>0.31743399999999999</v>
-      </c>
-      <c r="G14">
-        <v>0.316695</v>
-      </c>
-      <c r="H14">
-        <v>0.56482600000000005</v>
-      </c>
-      <c r="I14">
-        <v>0.87789099999999998</v>
-      </c>
-      <c r="J14">
-        <v>0.22776099999999999</v>
-      </c>
-      <c r="K14">
-        <v>156</v>
-      </c>
-      <c r="L14" t="s">
-        <v>36</v>
-      </c>
-      <c r="M14" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="15" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C15">
-        <v>12</v>
-      </c>
-      <c r="D15" t="s">
-        <v>2</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="C13" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="6">
+        <v>85.7</v>
+      </c>
+      <c r="G13" s="8">
+        <v>79.400000000000006</v>
+      </c>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F15">
-        <v>0.20847299999999999</v>
-      </c>
-      <c r="G15">
-        <v>0.19748199999999999</v>
-      </c>
-      <c r="H15">
-        <v>0.52421700000000004</v>
-      </c>
-      <c r="I15">
-        <v>0.64889399999999997</v>
-      </c>
-      <c r="J15">
-        <v>0.35109000000000001</v>
-      </c>
-      <c r="K15">
-        <v>156</v>
-      </c>
-      <c r="L15" t="s">
-        <v>36</v>
-      </c>
-      <c r="M15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C16">
-        <v>8</v>
-      </c>
-      <c r="D16" t="s">
-        <v>5</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="C14" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" s="6">
+        <v>64.5</v>
+      </c>
+      <c r="G14" s="8">
+        <v>63.2</v>
+      </c>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F16">
-        <v>0.26214500000000002</v>
-      </c>
-      <c r="G16">
-        <v>0.21366599999999999</v>
-      </c>
-      <c r="H16">
-        <v>0.67740699999999998</v>
-      </c>
-      <c r="I16">
-        <v>0.90226600000000001</v>
-      </c>
-      <c r="J16">
-        <v>0.312139</v>
-      </c>
-      <c r="K16">
-        <v>156</v>
-      </c>
-      <c r="L16" t="s">
-        <v>36</v>
-      </c>
-      <c r="M16" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C17">
-        <v>10</v>
-      </c>
-      <c r="D17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="C15" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="6">
+        <v>79.3</v>
+      </c>
+      <c r="G15" s="8">
+        <v>77.400000000000006</v>
+      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F17">
-        <v>0.24649599999999999</v>
-      </c>
-      <c r="G17">
-        <v>0.19878000000000001</v>
-      </c>
-      <c r="H17">
-        <v>0.96712799999999999</v>
-      </c>
-      <c r="I17">
-        <v>1.2556929999999999</v>
-      </c>
-      <c r="J17">
-        <v>0.32430199999999998</v>
-      </c>
-      <c r="K17">
-        <v>156</v>
-      </c>
-      <c r="L17" t="s">
-        <v>36</v>
-      </c>
-      <c r="M17" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C18">
-        <v>3</v>
-      </c>
-      <c r="D18" t="s">
-        <v>7</v>
-      </c>
-      <c r="E18" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18">
-        <v>0.45166200000000001</v>
-      </c>
-      <c r="G18">
-        <v>0.443276</v>
-      </c>
-      <c r="H18">
-        <v>1.084071</v>
-      </c>
-      <c r="I18">
-        <v>1.5324390000000001</v>
-      </c>
-      <c r="J18">
-        <v>0.266513</v>
-      </c>
-      <c r="K18">
-        <v>156</v>
-      </c>
-      <c r="L18" t="s">
-        <v>36</v>
-      </c>
-      <c r="M18" t="s">
-        <v>45</v>
+      <c r="C16" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" s="6">
+        <v>58.3</v>
+      </c>
+      <c r="G16" s="8">
+        <v>27.6</v>
+      </c>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F17" s="11">
+        <f>AVERAGE(F2,F5:F16)</f>
+        <v>73.284615384615378</v>
+      </c>
+      <c r="G17" s="11">
+        <f>AVERAGE(G2,G5:G16)</f>
+        <v>66.753846153846155</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C4:M18">
-    <sortCondition ref="E6:E18"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I16">
+    <sortCondition ref="B6:B16"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>